<commit_message>
Normalize chemical opened dates
</commit_message>
<xml_diff>
--- a/source/Inventory_Master_CategoryTabs_V4.xlsx
+++ b/source/Inventory_Master_CategoryTabs_V4.xlsx
@@ -628,7 +628,7 @@
         <x:v>RT</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>08.12.17</x:v>
+        <x:v>2008.12.17</x:v>
       </x:c>
       <x:c r="H11" s="12" t="str">
         <x:v>12.5ml</x:v>
@@ -1276,7 +1276,7 @@
         <x:v>RT</x:v>
       </x:c>
       <x:c r="G33" s="14" t="str">
-        <x:v>19.12.23</x:v>
+        <x:v>2019.12.23</x:v>
       </x:c>
       <x:c r="H33" s="12" t="str">
         <x:v>2g</x:v>
@@ -2239,7 +2239,7 @@
         <x:v>RT</x:v>
       </x:c>
       <x:c r="G66" s="14" t="str">
-        <x:v>12.10.19</x:v>
+        <x:v>2012.10.19</x:v>
       </x:c>
       <x:c r="H66" s="12" t="str">
         <x:v>10g</x:v>
@@ -2357,7 +2357,7 @@
         <x:v>RT</x:v>
       </x:c>
       <x:c r="G70" s="14" t="str">
-        <x:v>18.01.26</x:v>
+        <x:v>2018.01.26</x:v>
       </x:c>
       <x:c r="H70" s="12" t="str">
         <x:v>10g</x:v>
@@ -3005,7 +3005,7 @@
         <x:v>RT</x:v>
       </x:c>
       <x:c r="G92" s="14" t="str">
-        <x:v>09.08.27</x:v>
+        <x:v>2009.08.27</x:v>
       </x:c>
       <x:c r="H92" s="12" t="str">
         <x:v>250mg</x:v>
@@ -3473,7 +3473,7 @@
         <x:v>RT</x:v>
       </x:c>
       <x:c r="G108" s="14" t="str">
-        <x:v>10.07.07</x:v>
+        <x:v>2010.07.07</x:v>
       </x:c>
       <x:c r="H108" s="12" t="str">
         <x:v>1g</x:v>
@@ -3676,7 +3676,7 @@
         <x:v>RT</x:v>
       </x:c>
       <x:c r="G115" s="14" t="str">
-        <x:v>19.05.16</x:v>
+        <x:v>2019.05.16</x:v>
       </x:c>
       <x:c r="H115" s="12" t="str">
         <x:v>500g</x:v>
@@ -3736,7 +3736,7 @@
         <x:v>RT</x:v>
       </x:c>
       <x:c r="G117" s="14" t="str">
-        <x:v>19.05.16</x:v>
+        <x:v>2019.05.16</x:v>
       </x:c>
       <x:c r="H117" s="12" t="str">
         <x:v>500g</x:v>
@@ -4347,7 +4347,7 @@
         <x:v>RT</x:v>
       </x:c>
       <x:c r="G138" s="14" t="str">
-        <x:v>18.01.26</x:v>
+        <x:v>2018.01.26</x:v>
       </x:c>
       <x:c r="H138" s="12" t="str">
         <x:v>25g</x:v>
@@ -4970,7 +4970,7 @@
         <x:v>4'C</x:v>
       </x:c>
       <x:c r="G159" s="14" t="str">
-        <x:v>2010.07</x:v>
+        <x:v>2010.07.01</x:v>
       </x:c>
       <x:c r="H159" s="12" t="str">
         <x:v>150mL</x:v>

</xml_diff>

<commit_message>
Rename antibody requester column to note
</commit_message>
<xml_diff>
--- a/source/Inventory_Master_CategoryTabs_V4.xlsx
+++ b/source/Inventory_Master_CategoryTabs_V4.xlsx
@@ -11401,7 +11401,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K10" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -11434,7 +11434,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K11" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -11467,7 +11467,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K12" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -12225,7 +12225,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K38" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -12666,7 +12666,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K53" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -13134,7 +13134,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K69" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -13167,7 +13167,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K70" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -14132,7 +14132,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K103" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -15439,7 +15439,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K148" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -15501,7 +15501,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K150" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="151">
@@ -15592,7 +15592,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K153" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="154">
@@ -16058,7 +16058,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K169" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="170">
@@ -16438,7 +16438,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K181" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -16471,7 +16471,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K182" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -16591,7 +16591,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K186" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="187">
@@ -16653,7 +16653,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K188" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="189">
@@ -16744,7 +16744,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K191" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="192">
@@ -16974,7 +16974,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K199" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="200">
@@ -17092,7 +17092,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K203" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="204">
@@ -17154,7 +17154,7 @@
         <x:v>단종</x:v>
       </x:c>
       <x:c r="K205" s="12" t="str">
-        <x:v>단종</x:v>
+        <x:v/>
       </x:c>
     </x:row>
     <x:row r="206">

</xml_diff>

<commit_message>
Add CAS data to CategoryTabs inventory
</commit_message>
<xml_diff>
--- a/source/Inventory_Master_CategoryTabs_V4.xlsx
+++ b/source/Inventory_Master_CategoryTabs_V4.xlsx
@@ -10,7 +10,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217">
   <si>
     <t>Junsei</t>
   </si>
@@ -64,6 +64,603 @@
   </si>
   <si>
     <t>CST</t>
+  </si>
+  <si>
+    <t>CAS_No</t>
+  </si>
+  <si>
+    <t>152-11-4</t>
+  </si>
+  <si>
+    <t>97-00-7</t>
+  </si>
+  <si>
+    <t>7786-30-3</t>
+  </si>
+  <si>
+    <t>67-63-0</t>
+  </si>
+  <si>
+    <t>60-00-4</t>
+  </si>
+  <si>
+    <t>59-92-7</t>
+  </si>
+  <si>
+    <t>609-99-4</t>
+  </si>
+  <si>
+    <t>458-36-6</t>
+  </si>
+  <si>
+    <t>89-57-6</t>
+  </si>
+  <si>
+    <t>67-64-1</t>
+  </si>
+  <si>
+    <t>75-05-8</t>
+  </si>
+  <si>
+    <t>83-61-4</t>
+  </si>
+  <si>
+    <t>7446-70-0</t>
+  </si>
+  <si>
+    <t>7727-54-0</t>
+  </si>
+  <si>
+    <t>543-80-6</t>
+  </si>
+  <si>
+    <t>633-65-8</t>
+  </si>
+  <si>
+    <t>7659-95-2</t>
+  </si>
+  <si>
+    <t>331-39-5</t>
+  </si>
+  <si>
+    <t>10035-04-8</t>
+  </si>
+  <si>
+    <t>83881-52-1</t>
+  </si>
+  <si>
+    <t>123-03-5</t>
+  </si>
+  <si>
+    <t>94-41-7</t>
+  </si>
+  <si>
+    <t>67-66-3</t>
+  </si>
+  <si>
+    <t>327-97-9</t>
+  </si>
+  <si>
+    <t>7440-48-4</t>
+  </si>
+  <si>
+    <t>58367-01-4</t>
+  </si>
+  <si>
+    <t>30237-26-4</t>
+  </si>
+  <si>
+    <t>75-09-2</t>
+  </si>
+  <si>
+    <t>111-42-2</t>
+  </si>
+  <si>
+    <t>22494-42-4</t>
+  </si>
+  <si>
+    <t>67-68-5</t>
+  </si>
+  <si>
+    <t>64-17-5</t>
+  </si>
+  <si>
+    <t>33419-42-0</t>
+  </si>
+  <si>
+    <t>75-12-7</t>
+  </si>
+  <si>
+    <t>149-91-7</t>
+  </si>
+  <si>
+    <t>56-40-6</t>
+  </si>
+  <si>
+    <t>6004-24-6</t>
+  </si>
+  <si>
+    <t>7647-01-0</t>
+  </si>
+  <si>
+    <t>53-86-1</t>
+  </si>
+  <si>
+    <t>50-81-7</t>
+  </si>
+  <si>
+    <t>52-90-4</t>
+  </si>
+  <si>
+    <t>56-45-1</t>
+  </si>
+  <si>
+    <t>6080-56-4</t>
+  </si>
+  <si>
+    <t>7791-18-6</t>
+  </si>
+  <si>
+    <t>37267-86-0</t>
+  </si>
+  <si>
+    <t>67-56-1</t>
+  </si>
+  <si>
+    <t>1083299-87-9</t>
+  </si>
+  <si>
+    <t>1465-25-4</t>
+  </si>
+  <si>
+    <t>96829-58-2</t>
+  </si>
+  <si>
+    <t>501-98-4</t>
+  </si>
+  <si>
+    <t>57-10-3</t>
+  </si>
+  <si>
+    <t>329-98-6</t>
+  </si>
+  <si>
+    <t>7664-38-2</t>
+  </si>
+  <si>
+    <t>7447-40-7</t>
+  </si>
+  <si>
+    <t>6381-59-5</t>
+  </si>
+  <si>
+    <t>333-93-7</t>
+  </si>
+  <si>
+    <t>635-78-9</t>
+  </si>
+  <si>
+    <t>530-59-6</t>
+  </si>
+  <si>
+    <t>7784-46-5</t>
+  </si>
+  <si>
+    <t>144-55-8</t>
+  </si>
+  <si>
+    <t>497-19-8</t>
+  </si>
+  <si>
+    <t>9004-32-4</t>
+  </si>
+  <si>
+    <t>7647-14-5</t>
+  </si>
+  <si>
+    <t>151-21-3</t>
+  </si>
+  <si>
+    <t>1310-73-2</t>
+  </si>
+  <si>
+    <t>7681-57-4</t>
+  </si>
+  <si>
+    <t>7632-00-0</t>
+  </si>
+  <si>
+    <t>13721-39-6</t>
+  </si>
+  <si>
+    <t>7440-23-5</t>
+  </si>
+  <si>
+    <t>7558-79-4</t>
+  </si>
+  <si>
+    <t>7782-85-6</t>
+  </si>
+  <si>
+    <t>10102-18-8</t>
+  </si>
+  <si>
+    <t>7757-83-7</t>
+  </si>
+  <si>
+    <t>6106-24-7</t>
+  </si>
+  <si>
+    <t>57-50-1</t>
+  </si>
+  <si>
+    <t>63-74-1</t>
+  </si>
+  <si>
+    <t>7664-93-9</t>
+  </si>
+  <si>
+    <t>110-18-9</t>
+  </si>
+  <si>
+    <t>97-77-8</t>
+  </si>
+  <si>
+    <t>104-55-2</t>
+  </si>
+  <si>
+    <t>621-82-9</t>
+  </si>
+  <si>
+    <t>77-86-1</t>
+  </si>
+  <si>
+    <t>121-34-6</t>
+  </si>
+  <si>
+    <t>480-41-1</t>
+  </si>
+  <si>
+    <t>989-51-5</t>
+  </si>
+  <si>
+    <t>18457-55-1</t>
+  </si>
+  <si>
+    <t>88191-48-4</t>
+  </si>
+  <si>
+    <t>53188-07-1</t>
+  </si>
+  <si>
+    <t>122-31-6</t>
+  </si>
+  <si>
+    <t>1898-66-4</t>
+  </si>
+  <si>
+    <t>2997-92-4</t>
+  </si>
+  <si>
+    <t>610-02-6</t>
+  </si>
+  <si>
+    <t>99-96-7</t>
+  </si>
+  <si>
+    <t>87099-73-8</t>
+  </si>
+  <si>
+    <t>89886-31-7</t>
+  </si>
+  <si>
+    <t>57-06-7</t>
+  </si>
+  <si>
+    <t>592-88-1</t>
+  </si>
+  <si>
+    <t>5108-96-3</t>
+  </si>
+  <si>
+    <t>491-67-8</t>
+  </si>
+  <si>
+    <t>622-78-6</t>
+  </si>
+  <si>
+    <t>477-90-7</t>
+  </si>
+  <si>
+    <t>107-43-7</t>
+  </si>
+  <si>
+    <t>58-08-2</t>
+  </si>
+  <si>
+    <t>404-86-4</t>
+  </si>
+  <si>
+    <t>15663-27-1</t>
+  </si>
+  <si>
+    <t>35825-57-1</t>
+  </si>
+  <si>
+    <t>59865-13-3</t>
+  </si>
+  <si>
+    <t>47165-04-8</t>
+  </si>
+  <si>
+    <t>50-02-2</t>
+  </si>
+  <si>
+    <t>119-84-6</t>
+  </si>
+  <si>
+    <t>27565-41-9</t>
+  </si>
+  <si>
+    <t>25316-40-9</t>
+  </si>
+  <si>
+    <t>518-82-1</t>
+  </si>
+  <si>
+    <t>2002-24-6</t>
+  </si>
+  <si>
+    <t>97-53-0</t>
+  </si>
+  <si>
+    <t>518-17-2</t>
+  </si>
+  <si>
+    <t>64-18-6</t>
+  </si>
+  <si>
+    <t>548-83-4</t>
+  </si>
+  <si>
+    <t>520-33-2</t>
+  </si>
+  <si>
+    <t>700-06-1</t>
+  </si>
+  <si>
+    <t>146-68-9</t>
+  </si>
+  <si>
+    <t>56-86-0</t>
+  </si>
+  <si>
+    <t>70-18-8</t>
+  </si>
+  <si>
+    <t>108-95-2</t>
+  </si>
+  <si>
+    <t>28831-65-4</t>
+  </si>
+  <si>
+    <t>580-72-3</t>
+  </si>
+  <si>
+    <t>616-91-1</t>
+  </si>
+  <si>
+    <t>906-33-2</t>
+  </si>
+  <si>
+    <t>1405-10-3</t>
+  </si>
+  <si>
+    <t>64224-21-1</t>
+  </si>
+  <si>
+    <t>2257-09-2</t>
+  </si>
+  <si>
+    <t>36322-90-4</t>
+  </si>
+  <si>
+    <t>25535-16-4</t>
+  </si>
+  <si>
+    <t>129-56-6</t>
+  </si>
+  <si>
+    <t>480-18-2</t>
+  </si>
+  <si>
+    <t>85622-93-1</t>
+  </si>
+  <si>
+    <t>83-67-0</t>
+  </si>
+  <si>
+    <t>58-55-9</t>
+  </si>
+  <si>
+    <t>298-93-1</t>
+  </si>
+  <si>
+    <t>1135-24-6</t>
+  </si>
+  <si>
+    <t>77-52-1</t>
+  </si>
+  <si>
+    <t>97-16-5</t>
+  </si>
+  <si>
+    <t>522-17-8</t>
+  </si>
+  <si>
+    <t>490-83-5</t>
+  </si>
+  <si>
+    <t>32222-06-3</t>
+  </si>
+  <si>
+    <t>28822-58-4</t>
+  </si>
+  <si>
+    <t>1968-05-4</t>
+  </si>
+  <si>
+    <t>20525-20-6</t>
+  </si>
+  <si>
+    <t>5300-03-8</t>
+  </si>
+  <si>
+    <t>34369-07-8</t>
+  </si>
+  <si>
+    <t>136632-32-1</t>
+  </si>
+  <si>
+    <t>69-53-4</t>
+  </si>
+  <si>
+    <t>148504-34-1</t>
+  </si>
+  <si>
+    <t>70831-56-0</t>
+  </si>
+  <si>
+    <t>9001-12-1</t>
+  </si>
+  <si>
+    <t>458-37-7</t>
+  </si>
+  <si>
+    <t>1428-67-7</t>
+  </si>
+  <si>
+    <t>476-66-4</t>
+  </si>
+  <si>
+    <t>528-48-3</t>
+  </si>
+  <si>
+    <t>78824-30-3</t>
+  </si>
+  <si>
+    <t>446-72-0</t>
+  </si>
+  <si>
+    <t>5115-71-9</t>
+  </si>
+  <si>
+    <t>4091-99-0</t>
+  </si>
+  <si>
+    <t>1115-70-4</t>
+  </si>
+  <si>
+    <t>443-48-1</t>
+  </si>
+  <si>
+    <t>529-44-2</t>
+  </si>
+  <si>
+    <t>459789-99-2</t>
+  </si>
+  <si>
+    <t>112-80-1</t>
+  </si>
+  <si>
+    <t>20554-84-1</t>
+  </si>
+  <si>
+    <t>9013-05-2</t>
+  </si>
+  <si>
+    <t>57-83-0</t>
+  </si>
+  <si>
+    <t>53123-88-9</t>
+  </si>
+  <si>
+    <t>65666-07-1</t>
+  </si>
+  <si>
+    <t>131651-37-1</t>
+  </si>
+  <si>
+    <t>1404-93-9</t>
+  </si>
+  <si>
+    <t>133407-82-6</t>
+  </si>
+  <si>
+    <t>127-09-3</t>
+  </si>
+  <si>
+    <t>22055-22-7</t>
+  </si>
+  <si>
+    <t>18085-97-7</t>
+  </si>
+  <si>
+    <t>23027-91-0</t>
+  </si>
+  <si>
+    <t>50-00-0</t>
+  </si>
+  <si>
+    <t>5142-23-4</t>
+  </si>
+  <si>
+    <t>480-10-4</t>
+  </si>
+  <si>
+    <t>129453-61-8</t>
+  </si>
+  <si>
+    <t>173436-66-3</t>
+  </si>
+  <si>
+    <t>17912-87-7</t>
+  </si>
+  <si>
+    <t>301836-41-9</t>
+  </si>
+  <si>
+    <t>130-22-3</t>
+  </si>
+  <si>
+    <t>2802-68-8</t>
+  </si>
+  <si>
+    <t>9048-46-8</t>
+  </si>
+  <si>
+    <t>215-98-1</t>
+  </si>
+  <si>
+    <t>88899-55-2</t>
+  </si>
+  <si>
+    <t>11070-73-8</t>
+  </si>
+  <si>
+    <t>142825-10-3</t>
+  </si>
+  <si>
+    <t>9050-36-6</t>
+  </si>
+  <si>
+    <t>68424-85-1</t>
+  </si>
+  <si>
+    <t>75-91-2</t>
+  </si>
+  <si>
+    <t>9005-64-5</t>
   </si>
 </sst>
 </file>
@@ -397,6 +994,9 @@
       <c r="K1" s="6" t="str">
         <v>Note</v>
       </c>
+      <c r="L1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="str">
@@ -426,6 +1026,9 @@
       </c>
       <c r="J2" s="12"/>
       <c r="K2" s="12"/>
+      <c r="L2" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="str">
@@ -486,6 +1089,9 @@
       </c>
       <c r="J4" s="12"/>
       <c r="K4" s="12"/>
+      <c r="L4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="str">
@@ -544,6 +1150,9 @@
       </c>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
+      <c r="L6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="str">
@@ -662,6 +1271,9 @@
       </c>
       <c r="J10" s="12"/>
       <c r="K10" s="12"/>
+      <c r="L10" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="str">
@@ -693,6 +1305,9 @@
       </c>
       <c r="J11" s="12"/>
       <c r="K11" s="12"/>
+      <c r="L11" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="str">
@@ -722,6 +1337,9 @@
       </c>
       <c r="J12" s="12"/>
       <c r="K12" s="12"/>
+      <c r="L12" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="str">
@@ -751,6 +1369,9 @@
       </c>
       <c r="J13" s="12"/>
       <c r="K13" s="12"/>
+      <c r="L13" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="str">
@@ -780,6 +1401,9 @@
       </c>
       <c r="J14" s="12"/>
       <c r="K14" s="12"/>
+      <c r="L14" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="str">
@@ -840,6 +1464,9 @@
       </c>
       <c r="J16" s="12"/>
       <c r="K16" s="12"/>
+      <c r="L16" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="str">
@@ -958,6 +1585,9 @@
       </c>
       <c r="J20" s="12"/>
       <c r="K20" s="12"/>
+      <c r="L20" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="str">
@@ -987,6 +1617,9 @@
       </c>
       <c r="J21" s="12"/>
       <c r="K21" s="12"/>
+      <c r="L21" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="str">
@@ -1105,6 +1738,9 @@
       </c>
       <c r="J25" s="12"/>
       <c r="K25" s="12"/>
+      <c r="L25" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="str">
@@ -1134,6 +1770,9 @@
       </c>
       <c r="J26" s="12"/>
       <c r="K26" s="12"/>
+      <c r="L26" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="str">
@@ -1163,6 +1802,9 @@
       </c>
       <c r="J27" s="12"/>
       <c r="K27" s="12"/>
+      <c r="L27" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="str">
@@ -1221,6 +1863,9 @@
       </c>
       <c r="J29" s="12"/>
       <c r="K29" s="12"/>
+      <c r="L29" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="str">
@@ -1250,6 +1895,9 @@
       </c>
       <c r="J30" s="12"/>
       <c r="K30" s="12"/>
+      <c r="L30" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="str">
@@ -1281,6 +1929,9 @@
       </c>
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
+      <c r="L31" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="12" t="str">
@@ -1310,6 +1961,9 @@
       </c>
       <c r="J32" s="12"/>
       <c r="K32" s="12"/>
+      <c r="L32" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="str">
@@ -1341,6 +1995,9 @@
       </c>
       <c r="J33" s="12"/>
       <c r="K33" s="12"/>
+      <c r="L33" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="str">
@@ -1370,6 +2027,9 @@
       </c>
       <c r="J34" s="12"/>
       <c r="K34" s="12"/>
+      <c r="L34" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="str">
@@ -1399,6 +2059,9 @@
       </c>
       <c r="J35" s="12"/>
       <c r="K35" s="12"/>
+      <c r="L35" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="str">
@@ -1428,6 +2091,9 @@
       </c>
       <c r="J36" s="12"/>
       <c r="K36" s="12"/>
+      <c r="L36" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="str">
@@ -1457,6 +2123,9 @@
       </c>
       <c r="J37" s="12"/>
       <c r="K37" s="12"/>
+      <c r="L37" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="12" t="str">
@@ -1486,6 +2155,9 @@
       </c>
       <c r="J38" s="12"/>
       <c r="K38" s="12"/>
+      <c r="L38" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="str">
@@ -1515,6 +2187,9 @@
       </c>
       <c r="J39" s="12"/>
       <c r="K39" s="12"/>
+      <c r="L39" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="12" t="str">
@@ -1575,6 +2250,9 @@
       </c>
       <c r="J41" s="12"/>
       <c r="K41" s="12"/>
+      <c r="L41" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="12" t="str">
@@ -1633,6 +2311,9 @@
       </c>
       <c r="J43" s="12"/>
       <c r="K43" s="12"/>
+      <c r="L43" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="12" t="str">
@@ -1662,6 +2343,9 @@
       </c>
       <c r="J44" s="12"/>
       <c r="K44" s="12"/>
+      <c r="L44" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="12" t="str">
@@ -1691,6 +2375,9 @@
       </c>
       <c r="J45" s="12"/>
       <c r="K45" s="12"/>
+      <c r="L45" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="str">
@@ -1778,6 +2465,9 @@
       </c>
       <c r="J48" s="12"/>
       <c r="K48" s="12"/>
+      <c r="L48" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="str">
@@ -1807,6 +2497,9 @@
       </c>
       <c r="J49" s="12"/>
       <c r="K49" s="12"/>
+      <c r="L49" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="str">
@@ -1894,6 +2587,9 @@
       </c>
       <c r="J52" s="12"/>
       <c r="K52" s="12"/>
+      <c r="L52" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="str">
@@ -1923,6 +2619,9 @@
       </c>
       <c r="J53" s="12"/>
       <c r="K53" s="12"/>
+      <c r="L53" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="str">
@@ -1952,6 +2651,9 @@
       </c>
       <c r="J54" s="12"/>
       <c r="K54" s="12"/>
+      <c r="L54" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="12" t="str">
@@ -2010,6 +2712,9 @@
       </c>
       <c r="J56" s="12"/>
       <c r="K56" s="12"/>
+      <c r="L56" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="12" t="str">
@@ -2039,6 +2744,9 @@
       </c>
       <c r="J57" s="12"/>
       <c r="K57" s="12"/>
+      <c r="L57" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="12" t="str">
@@ -2068,6 +2776,9 @@
       </c>
       <c r="J58" s="12"/>
       <c r="K58" s="12"/>
+      <c r="L58" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="12" t="str">
@@ -2126,6 +2837,9 @@
       </c>
       <c r="J60" s="12"/>
       <c r="K60" s="12"/>
+      <c r="L60" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="str">
@@ -2244,6 +2958,9 @@
       </c>
       <c r="J64" s="12"/>
       <c r="K64" s="12"/>
+      <c r="L64" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="12" t="str">
@@ -2273,6 +2990,9 @@
       </c>
       <c r="J65" s="12"/>
       <c r="K65" s="12"/>
+      <c r="L65" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="12" t="str">
@@ -2304,6 +3024,9 @@
       </c>
       <c r="J66" s="12"/>
       <c r="K66" s="12"/>
+      <c r="L66" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="12" t="str">
@@ -2391,6 +3114,9 @@
       </c>
       <c r="J69" s="12"/>
       <c r="K69" s="12"/>
+      <c r="L69" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="12" t="str">
@@ -2480,6 +3206,9 @@
       </c>
       <c r="J72" s="12"/>
       <c r="K72" s="12"/>
+      <c r="L72" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="str">
@@ -2538,6 +3267,9 @@
       </c>
       <c r="J74" s="12"/>
       <c r="K74" s="12"/>
+      <c r="L74" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="str">
@@ -2596,6 +3328,9 @@
       </c>
       <c r="J76" s="12"/>
       <c r="K76" s="12"/>
+      <c r="L76" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="str">
@@ -2654,6 +3389,9 @@
       </c>
       <c r="J78" s="12"/>
       <c r="K78" s="12"/>
+      <c r="L78" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="str">
@@ -2714,6 +3452,9 @@
       </c>
       <c r="J80" s="12"/>
       <c r="K80" s="12"/>
+      <c r="L80" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="12" t="str">
@@ -2743,6 +3484,9 @@
       </c>
       <c r="J81" s="12"/>
       <c r="K81" s="12"/>
+      <c r="L81" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="str">
@@ -2772,6 +3516,9 @@
       </c>
       <c r="J82" s="12"/>
       <c r="K82" s="12"/>
+      <c r="L82" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="12" t="str">
@@ -2801,6 +3548,9 @@
       </c>
       <c r="J83" s="12"/>
       <c r="K83" s="12"/>
+      <c r="L83" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="str">
@@ -2863,6 +3613,9 @@
       </c>
       <c r="J85" s="12"/>
       <c r="K85" s="12"/>
+      <c r="L85" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="12" t="str">
@@ -2892,6 +3645,9 @@
       </c>
       <c r="J86" s="12"/>
       <c r="K86" s="12"/>
+      <c r="L86" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="str">
@@ -2921,6 +3677,9 @@
       </c>
       <c r="J87" s="12"/>
       <c r="K87" s="12"/>
+      <c r="L87" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="str">
@@ -2950,6 +3709,9 @@
       </c>
       <c r="J88" s="12"/>
       <c r="K88" s="12"/>
+      <c r="L88" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="str">
@@ -2981,6 +3743,9 @@
       </c>
       <c r="J89" s="12"/>
       <c r="K89" s="12"/>
+      <c r="L89" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="12" t="str">
@@ -3010,6 +3775,9 @@
       </c>
       <c r="J90" s="12"/>
       <c r="K90" s="12"/>
+      <c r="L90" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="12" t="str">
@@ -3039,6 +3807,9 @@
       </c>
       <c r="J91" s="12"/>
       <c r="K91" s="12"/>
+      <c r="L91" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="12" t="str">
@@ -3070,6 +3841,9 @@
       </c>
       <c r="J92" s="12"/>
       <c r="K92" s="12"/>
+      <c r="L92" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="12" t="str">
@@ -3099,6 +3873,9 @@
       </c>
       <c r="J93" s="12"/>
       <c r="K93" s="12"/>
+      <c r="L93" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="12" t="str">
@@ -3215,6 +3992,9 @@
       </c>
       <c r="J97" s="12"/>
       <c r="K97" s="12"/>
+      <c r="L97" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="12" t="str">
@@ -3244,6 +4024,9 @@
       </c>
       <c r="J98" s="12"/>
       <c r="K98" s="12"/>
+      <c r="L98" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="12" t="str">
@@ -3275,6 +4058,9 @@
       </c>
       <c r="J99" s="12"/>
       <c r="K99" s="12"/>
+      <c r="L99" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="12" t="str">
@@ -3304,6 +4090,9 @@
       </c>
       <c r="J100" s="12"/>
       <c r="K100" s="12"/>
+      <c r="L100" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="12" t="str">
@@ -3333,6 +4122,9 @@
       </c>
       <c r="J101" s="12"/>
       <c r="K101" s="12"/>
+      <c r="L101" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="12" t="str">
@@ -3420,6 +4212,9 @@
       </c>
       <c r="J104" s="12"/>
       <c r="K104" s="12"/>
+      <c r="L104" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="12" t="str">
@@ -3449,6 +4244,9 @@
       </c>
       <c r="J105" s="12"/>
       <c r="K105" s="12"/>
+      <c r="L105" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="12" t="str">
@@ -3478,6 +4276,9 @@
       </c>
       <c r="J106" s="12"/>
       <c r="K106" s="12"/>
+      <c r="L106" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="12" t="str">
@@ -3538,6 +4339,9 @@
       </c>
       <c r="J108" s="12"/>
       <c r="K108" s="12"/>
+      <c r="L108" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="12" t="str">
@@ -3652,6 +4456,9 @@
       </c>
       <c r="J112" s="12"/>
       <c r="K112" s="12"/>
+      <c r="L112" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="12" t="str">
@@ -3681,6 +4488,9 @@
       </c>
       <c r="J113" s="12"/>
       <c r="K113" s="12"/>
+      <c r="L113" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="12" t="str">
@@ -3710,6 +4520,9 @@
       </c>
       <c r="J114" s="12"/>
       <c r="K114" s="12"/>
+      <c r="L114" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="12" t="str">
@@ -3741,6 +4554,9 @@
       </c>
       <c r="J115" s="12"/>
       <c r="K115" s="12"/>
+      <c r="L115" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="12" t="str">
@@ -3770,6 +4586,9 @@
       </c>
       <c r="J116" s="12"/>
       <c r="K116" s="12"/>
+      <c r="L116" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="12" t="str">
@@ -3801,6 +4620,9 @@
       </c>
       <c r="J117" s="12"/>
       <c r="K117" s="12"/>
+      <c r="L117" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="12" t="str">
@@ -3830,6 +4652,9 @@
       </c>
       <c r="J118" s="12"/>
       <c r="K118" s="12"/>
+      <c r="L118" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="12" t="str">
@@ -3859,6 +4684,9 @@
       </c>
       <c r="J119" s="12"/>
       <c r="K119" s="12"/>
+      <c r="L119" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="12" t="str">
@@ -3888,6 +4716,9 @@
       </c>
       <c r="J120" s="12"/>
       <c r="K120" s="12"/>
+      <c r="L120" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="12" t="str">
@@ -3917,6 +4748,9 @@
       </c>
       <c r="J121" s="12"/>
       <c r="K121" s="12"/>
+      <c r="L121" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="12" t="str">
@@ -3946,6 +4780,9 @@
       </c>
       <c r="J122" s="12"/>
       <c r="K122" s="12"/>
+      <c r="L122" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="12" t="str">
@@ -4004,6 +4841,9 @@
       </c>
       <c r="J124" s="12"/>
       <c r="K124" s="12"/>
+      <c r="L124" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="12" t="str">
@@ -4035,6 +4875,9 @@
       </c>
       <c r="J125" s="12"/>
       <c r="K125" s="12"/>
+      <c r="L125" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="12" t="str">
@@ -4064,6 +4907,9 @@
       </c>
       <c r="J126" s="12"/>
       <c r="K126" s="12"/>
+      <c r="L126" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="12" t="str">
@@ -4093,6 +4939,9 @@
       </c>
       <c r="J127" s="12"/>
       <c r="K127" s="12"/>
+      <c r="L127" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="12" t="str">
@@ -4122,6 +4971,9 @@
       </c>
       <c r="J128" s="12"/>
       <c r="K128" s="12"/>
+      <c r="L128" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="12" t="str">
@@ -4151,6 +5003,9 @@
       </c>
       <c r="J129" s="12"/>
       <c r="K129" s="12"/>
+      <c r="L129" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="12" t="str">
@@ -4180,6 +5035,9 @@
       </c>
       <c r="J130" s="12"/>
       <c r="K130" s="12"/>
+      <c r="L130" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="12" t="str">
@@ -4209,6 +5067,9 @@
       </c>
       <c r="J131" s="12"/>
       <c r="K131" s="12"/>
+      <c r="L131" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="12" t="str">
@@ -4238,6 +5099,9 @@
       </c>
       <c r="J132" s="12"/>
       <c r="K132" s="12"/>
+      <c r="L132" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="12" t="str">
@@ -4265,6 +5129,9 @@
       </c>
       <c r="J133" s="12"/>
       <c r="K133" s="12"/>
+      <c r="L133" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="12" t="str">
@@ -4294,6 +5161,9 @@
       </c>
       <c r="J134" s="12"/>
       <c r="K134" s="12"/>
+      <c r="L134" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="12" t="str">
@@ -4323,6 +5193,9 @@
       </c>
       <c r="J135" s="12"/>
       <c r="K135" s="12"/>
+      <c r="L135" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="12" t="str">
@@ -4352,6 +5225,9 @@
       </c>
       <c r="J136" s="12"/>
       <c r="K136" s="12"/>
+      <c r="L136" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="12" t="str">
@@ -4381,6 +5257,9 @@
       </c>
       <c r="J137" s="12"/>
       <c r="K137" s="12"/>
+      <c r="L137" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="12" t="str">
@@ -4412,6 +5291,9 @@
       </c>
       <c r="J138" s="12"/>
       <c r="K138" s="12"/>
+      <c r="L138" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="12" t="str">
@@ -4441,6 +5323,9 @@
       </c>
       <c r="J139" s="12"/>
       <c r="K139" s="12"/>
+      <c r="L139" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="12" t="str">
@@ -4470,6 +5355,9 @@
       </c>
       <c r="J140" s="12"/>
       <c r="K140" s="12"/>
+      <c r="L140" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="12" t="str">
@@ -4644,6 +5532,9 @@
       </c>
       <c r="J146" s="12"/>
       <c r="K146" s="12"/>
+      <c r="L146" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="12" t="str">
@@ -4816,6 +5707,9 @@
       </c>
       <c r="J152" s="12"/>
       <c r="K152" s="12"/>
+      <c r="L152" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="12" t="str">
@@ -4847,6 +5741,9 @@
       <c r="K153" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L153" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="12" t="str">
@@ -4880,6 +5777,9 @@
       <c r="K154" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L154" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="12" t="str">
@@ -4911,6 +5811,9 @@
       <c r="K155" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L155" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="12" t="str">
@@ -4942,6 +5845,9 @@
       <c r="K156" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L156" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="12" t="str">
@@ -5004,6 +5910,9 @@
       <c r="K158" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L158" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="12" t="str">
@@ -5068,6 +5977,9 @@
       <c r="K160" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L160" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="12" t="str">
@@ -5165,6 +6077,9 @@
       <c r="K163" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L163" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="12" t="str">
@@ -5198,6 +6113,9 @@
       <c r="K164" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L164" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="12" t="str">
@@ -5262,6 +6180,9 @@
       <c r="K166" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L166" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="12" t="str">
@@ -5293,6 +6214,9 @@
       <c r="K167" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L167" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="12" t="str">
@@ -5324,6 +6248,9 @@
       <c r="K168" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L168" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="12" t="str">
@@ -5514,6 +6441,9 @@
       <c r="K174" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L174" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="12" t="str">
@@ -5545,6 +6475,9 @@
       <c r="K175" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L175" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="12" t="str">
@@ -5576,6 +6509,9 @@
       <c r="K176" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L176" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="12" t="str">
@@ -5609,6 +6545,9 @@
       <c r="K177" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L177" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="12" t="str">
@@ -5640,6 +6579,9 @@
       <c r="K178" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L178" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="12" t="str">
@@ -5671,6 +6613,9 @@
       <c r="K179" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L179" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="12" t="str">
@@ -5704,6 +6649,9 @@
       <c r="K180" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L180" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="12" t="str">
@@ -5766,6 +6714,9 @@
       <c r="K182" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L182" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="12" t="str">
@@ -5799,6 +6750,9 @@
       <c r="K183" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L183" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="12" t="str">
@@ -5892,6 +6846,9 @@
       <c r="K186" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L186" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="12" t="str">
@@ -5954,6 +6911,9 @@
       <c r="K188" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L188" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="12" t="str">
@@ -5985,6 +6945,9 @@
       <c r="K189" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L189" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="12" t="str">
@@ -6049,6 +7012,9 @@
       <c r="K191" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L191" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="12" t="str">
@@ -6080,6 +7046,9 @@
       <c r="K192" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L192" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="12" t="str">
@@ -6111,6 +7080,9 @@
       <c r="K193" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L193" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="12" t="str">
@@ -6142,6 +7114,9 @@
       <c r="K194" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L194" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="12" t="str">
@@ -6173,6 +7148,9 @@
       <c r="K195" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L195" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="12" t="str">
@@ -6266,6 +7244,9 @@
       <c r="K198" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L198" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="12" t="str">
@@ -6295,6 +7276,9 @@
       <c r="K199" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L199" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="12" t="str">
@@ -6326,6 +7310,9 @@
       <c r="K200" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L200" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="12" t="str">
@@ -6359,6 +7346,9 @@
       <c r="K201" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L201" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="12" t="str">
@@ -6392,6 +7382,9 @@
       <c r="K202" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L202" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="12" t="str">
@@ -6423,6 +7416,9 @@
       <c r="K203" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L203" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="12" t="str">
@@ -6456,6 +7452,9 @@
       <c r="K204" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L204" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="12" t="str">
@@ -6642,6 +7641,9 @@
       <c r="K210" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L210" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="12" t="str">
@@ -6735,6 +7737,9 @@
       <c r="K213" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L213" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="12" t="str">
@@ -6768,6 +7773,9 @@
       <c r="K214" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L214" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="12" t="str">
@@ -6832,6 +7840,9 @@
       <c r="K216" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L216" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="12" t="str">
@@ -6894,6 +7905,9 @@
       <c r="K218" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L218" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="12" t="str">
@@ -6956,6 +7970,9 @@
       <c r="K220" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L220" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="12" t="str">
@@ -6987,6 +8004,9 @@
       <c r="K221" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L221" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="12" t="str">
@@ -7048,6 +8068,9 @@
       <c r="J223" s="12"/>
       <c r="K223" s="12" t="str">
         <v>Ref #4</v>
+      </c>
+      <c r="L223" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="224">
@@ -7207,6 +8230,9 @@
       <c r="K228" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L228" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="12" t="str">
@@ -7238,6 +8264,9 @@
       <c r="K229" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L229" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="12" t="str">
@@ -7269,6 +8298,9 @@
       <c r="K230" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L230" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="12" t="str">
@@ -7364,6 +8396,9 @@
       <c r="K233" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L233" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="12" t="str">
@@ -7395,6 +8430,9 @@
       <c r="K234" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L234" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="12" t="str">
@@ -7428,6 +8466,9 @@
       <c r="K235" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L235" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="12" t="str">
@@ -7494,6 +8535,9 @@
       <c r="K237" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L237" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="12" t="str">
@@ -7556,6 +8600,9 @@
       <c r="K239" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L239" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="12" t="str">
@@ -7617,6 +8664,9 @@
       <c r="J241" s="12"/>
       <c r="K241" s="12" t="str">
         <v>Ref #4</v>
+      </c>
+      <c r="L241" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="242">
@@ -7897,6 +8947,9 @@
       <c r="K250" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L250" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="12" t="str">
@@ -8056,6 +9109,9 @@
       <c r="K255" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L255" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="12" t="str">
@@ -8087,6 +9143,9 @@
       <c r="K256" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L256" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="12" t="str">
@@ -8151,6 +9210,9 @@
       <c r="K258" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L258" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="12" t="str">
@@ -8182,6 +9244,9 @@
       <c r="K259" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L259" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="12" t="str">
@@ -8213,6 +9278,9 @@
       <c r="K260" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L260" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="12" t="str">
@@ -8246,6 +9314,9 @@
       <c r="K261" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L261" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="12" t="str">
@@ -8277,6 +9348,9 @@
       <c r="K262" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L262" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="12" t="str">
@@ -8308,6 +9382,9 @@
       <c r="K263" s="12" t="str">
         <v>Ref #4</v>
       </c>
+      <c r="L263" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="12" t="str">
@@ -8341,6 +9418,9 @@
       <c r="K264" s="12" t="str">
         <v>Ref #3</v>
       </c>
+      <c r="L264" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="12" t="str">
@@ -8839,6 +9919,9 @@
       <c r="K280" s="12" t="str">
         <v>Ref #6</v>
       </c>
+      <c r="L280" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="12" t="str">
@@ -8901,6 +9984,9 @@
       <c r="K282" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L282" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="12" t="str">
@@ -8932,6 +10018,9 @@
       <c r="K283" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L283" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="12" t="str">
@@ -8963,6 +10052,9 @@
       <c r="K284" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L284" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="12" t="str">
@@ -8994,6 +10086,9 @@
       <c r="K285" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L285" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="12" t="str">
@@ -9025,6 +10120,9 @@
       <c r="K286" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L286" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="12" t="str">
@@ -9056,6 +10154,9 @@
       <c r="K287" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L287" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="12" t="str">
@@ -9087,6 +10188,9 @@
       <c r="K288" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L288" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="12" t="str">
@@ -9118,6 +10222,9 @@
       <c r="K289" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L289" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="12" t="str">
@@ -9273,6 +10380,9 @@
       <c r="K294" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L294" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="12" t="str">
@@ -9304,6 +10414,9 @@
       <c r="K295" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L295" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="12" t="str">
@@ -9366,6 +10479,9 @@
       <c r="K297" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L297" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="12" t="str">
@@ -9397,6 +10513,9 @@
       <c r="K298" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L298" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="12" t="str">
@@ -9428,6 +10547,9 @@
       <c r="K299" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L299" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="12" t="str">
@@ -9490,6 +10612,9 @@
       <c r="K301" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L301" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="12" t="str">
@@ -9583,6 +10708,9 @@
       <c r="K304" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L304" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="12" t="str">
@@ -9614,6 +10742,9 @@
       <c r="K305" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L305" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="12" t="str">
@@ -9676,6 +10807,9 @@
       <c r="K307" s="12" t="str">
         <v>Fridge #2</v>
       </c>
+      <c r="L307" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="12" t="str">
@@ -9707,6 +10841,9 @@
       <c r="K308" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L308" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="12" t="str">
@@ -9738,6 +10875,9 @@
       <c r="K309" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L309" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="12" t="str">
@@ -9769,6 +10909,9 @@
       <c r="K310" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L310" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="12" t="str">
@@ -9800,6 +10943,9 @@
       <c r="K311" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L311" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="12" t="str">
@@ -9831,6 +10977,9 @@
       <c r="K312" s="12" t="str">
         <v>Fridge #2</v>
       </c>
+      <c r="L312" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="12" t="str">
@@ -9862,6 +11011,9 @@
       <c r="K313" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L313" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="12" t="str">
@@ -10048,6 +11200,9 @@
       <c r="K319" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L319" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="12" t="str">
@@ -10079,6 +11234,9 @@
       <c r="K320" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L320" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="12" t="str">
@@ -10141,6 +11299,9 @@
       <c r="K322" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L322" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="12" t="str">
@@ -10172,6 +11333,9 @@
       <c r="K323" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L323" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="12" t="str">
@@ -10203,6 +11367,9 @@
       <c r="K324" s="12" t="str">
         <v>Fridge #2</v>
       </c>
+      <c r="L324" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="12" t="str">
@@ -10234,6 +11401,9 @@
       <c r="K325" s="12" t="str">
         <v>Fridge #2</v>
       </c>
+      <c r="L325" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="12" t="str">
@@ -10265,6 +11435,9 @@
       <c r="K326" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L326" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="12" t="str">
@@ -10327,6 +11500,9 @@
       <c r="K328" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L328" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="12" t="str">
@@ -10358,6 +11534,9 @@
       <c r="K329" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L329" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="12" t="str">
@@ -10451,6 +11630,9 @@
       <c r="K332" s="12" t="str">
         <v>Fridge #5</v>
       </c>
+      <c r="L332" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="12" t="str">
@@ -10575,6 +11757,9 @@
       <c r="K336" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L336" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="12" t="str">
@@ -10730,6 +11915,9 @@
       <c r="K341" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L341" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="12" t="str">
@@ -10792,6 +11980,9 @@
       <c r="K343" s="12" t="str">
         <v>Fridge #7</v>
       </c>
+      <c r="L343" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="12" t="str">
@@ -10822,6 +12013,9 @@
       <c r="J344" s="12"/>
       <c r="K344" s="12" t="str">
         <v>Fridge #5</v>
+      </c>
+      <c r="L344" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="345">
@@ -20658,6 +21852,9 @@
       <c r="F1" s="6" t="str">
         <v>Storage</v>
       </c>
+      <c r="G1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="str">
@@ -20792,6 +21989,9 @@
         <v>A13184.0B</v>
       </c>
       <c r="F8" s="12"/>
+      <c r="G8" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="str">
@@ -20812,6 +22012,9 @@
       <c r="F9" s="12" t="str">
         <v>RT</v>
       </c>
+      <c r="G9" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="str">
@@ -21242,6 +22445,9 @@
       <c r="F32" s="12" t="str">
         <v>4℃</v>
       </c>
+      <c r="G32" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="str">
@@ -21262,6 +22468,9 @@
       <c r="F33" s="12" t="str">
         <v>4℃</v>
       </c>
+      <c r="G33" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="str">
@@ -21282,6 +22491,9 @@
       <c r="F34" s="12" t="str">
         <v>4℃</v>
       </c>
+      <c r="G34" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="str">
@@ -22214,6 +23426,9 @@
       <c r="F83" s="12" t="str">
         <v>RT</v>
       </c>
+      <c r="G83" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="str">
@@ -22292,6 +23507,9 @@
         <v>HY-19312-50mg</v>
       </c>
       <c r="F87" s="12"/>
+      <c r="G87" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="str">
@@ -22312,6 +23530,9 @@
       <c r="F88" s="12" t="str">
         <v>4℃</v>
       </c>
+      <c r="G88" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="str">
@@ -22332,6 +23553,9 @@
       <c r="F89" s="12" t="str">
         <v>4°C</v>
       </c>
+      <c r="G89" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="12" t="str">
@@ -22352,6 +23576,9 @@
       <c r="F90" s="12" t="str">
         <v>4℃</v>
       </c>
+      <c r="G90" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="12" t="str">
@@ -22372,6 +23599,9 @@
       <c r="F91" s="12" t="str">
         <v>4℃</v>
       </c>
+      <c r="G91" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="12" t="str">
@@ -22392,6 +23622,9 @@
       <c r="F92" s="12" t="str">
         <v>4℃</v>
       </c>
+      <c r="G92" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="12" t="str">
@@ -22410,6 +23643,9 @@
         <v>HY-10219-10mg</v>
       </c>
       <c r="F93" s="12"/>
+      <c r="G93" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="12" t="str">
@@ -22430,6 +23666,9 @@
       <c r="F94" s="12" t="str">
         <v>4℃</v>
       </c>
+      <c r="G94" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="12" t="str">
@@ -23118,6 +24357,9 @@
         <v>A5533-25g</v>
       </c>
       <c r="F131" s="12"/>
+      <c r="G131" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="12" t="str">
@@ -23136,6 +24378,9 @@
         <v>61626-1L</v>
       </c>
       <c r="F132" s="12"/>
+      <c r="G132" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="12" t="str">
@@ -23156,6 +24401,9 @@
       <c r="F133" s="12" t="str">
         <v>4℃</v>
       </c>
+      <c r="G133" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="12" t="str">
@@ -23176,6 +24424,9 @@
       <c r="F134" s="12" t="str">
         <v>RT</v>
       </c>
+      <c r="G134" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="12" t="str">
@@ -23216,6 +24467,9 @@
       <c r="F136" s="12" t="str">
         <v>RT</v>
       </c>
+      <c r="G136" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="12" t="str">
@@ -23236,6 +24490,9 @@
       <c r="F137" s="12" t="str">
         <v>-20℃</v>
       </c>
+      <c r="G137" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="12" t="str">
@@ -23256,6 +24513,9 @@
       <c r="F138" s="12" t="str">
         <v>-20°C</v>
       </c>
+      <c r="G138" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="12" t="str">
@@ -23296,6 +24556,9 @@
       <c r="F140" s="12" t="str">
         <v>-20°C</v>
       </c>
+      <c r="G140" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="12" t="str">
@@ -23314,6 +24577,9 @@
         <v>419680-100g</v>
       </c>
       <c r="F141" s="12"/>
+      <c r="G141" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="12" t="str">
@@ -23332,6 +24598,9 @@
         <v>419680-500g</v>
       </c>
       <c r="F142" s="12"/>
+      <c r="G142" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="12" t="str">
@@ -23352,6 +24621,9 @@
       <c r="F143" s="12" t="str">
         <v>4℃</v>
       </c>
+      <c r="G143" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="str">
@@ -23370,6 +24642,9 @@
         <v>P7626-1g</v>
       </c>
       <c r="F144" s="12"/>
+      <c r="G144" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="12" t="str">
@@ -23388,6 +24663,9 @@
         <v>S5525-4OZ</v>
       </c>
       <c r="F145" s="12"/>
+      <c r="G145" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="12" t="str">
@@ -23406,6 +24684,9 @@
         <v>458139-25mL</v>
       </c>
       <c r="F146" s="12"/>
+      <c r="G146" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="12" t="str">
@@ -23446,6 +24727,9 @@
       <c r="F148" s="12" t="str">
         <v>RT</v>
       </c>
+      <c r="G148" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="12" t="str">
@@ -23464,6 +24748,9 @@
         <v>SM-GLC-001</v>
       </c>
       <c r="F149" s="12"/>
+      <c r="G149" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="12" t="str">
@@ -23484,6 +24771,9 @@
       <c r="F150" s="12" t="str">
         <v>RT</v>
       </c>
+      <c r="G150" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="12" t="str">
@@ -23754,6 +25044,9 @@
         <v>109634.1011</v>
       </c>
       <c r="F165" s="12"/>
+      <c r="G165" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="12" t="str">
@@ -23772,6 +25065,9 @@
         <v>100983.1011</v>
       </c>
       <c r="F166" s="12"/>
+      <c r="G166" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="12" t="str">
@@ -23790,6 +25086,9 @@
         <v>106009.1011</v>
       </c>
       <c r="F167" s="12"/>
+      <c r="G167" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="12" t="str">
@@ -23810,6 +25109,9 @@
       <c r="F168" s="12" t="str">
         <v>2-30°C</v>
       </c>
+      <c r="G168" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="12" t="str">
@@ -24300,6 +25602,9 @@
         <v>4095-3705</v>
       </c>
       <c r="F194" s="12"/>
+      <c r="G194" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="12" t="str">
@@ -24318,6 +25623,9 @@
         <v>4097-3700</v>
       </c>
       <c r="F195" s="12"/>
+      <c r="G195" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="12" t="str">
@@ -24336,6 +25644,9 @@
         <v>4204-4410</v>
       </c>
       <c r="F196" s="12"/>
+      <c r="G196" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="12" t="str">
@@ -24354,6 +25665,9 @@
         <v>5558-4410</v>
       </c>
       <c r="F197" s="12"/>
+      <c r="G197" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="12" t="str">

</xml_diff>

<commit_message>
Normalize Chemical Biacore manufacturer
</commit_message>
<xml_diff>
--- a/source/Inventory_Master_CategoryTabs_V4.xlsx
+++ b/source/Inventory_Master_CategoryTabs_V4.xlsx
@@ -10,7 +10,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="218">
   <si>
     <t>Junsei</t>
   </si>
@@ -662,6 +662,9 @@
   <si>
     <t>9005-64-5</t>
   </si>
+  <si>
+    <t>Cytiva</t>
+  </si>
 </sst>
 </file>
 
@@ -6260,7 +6263,7 @@
         <v>CHM-0168</v>
       </c>
       <c r="C169" s="12" t="s">
-        <v>7</v>
+        <v>217</v>
       </c>
       <c r="D169" s="12" t="str">
         <v>Acetate 4.0</v>
@@ -6291,7 +6294,7 @@
         <v>CHM-0169</v>
       </c>
       <c r="C170" s="12" t="s">
-        <v>7</v>
+        <v>217</v>
       </c>
       <c r="D170" s="12" t="str">
         <v>Acetate 4.5</v>
@@ -6322,7 +6325,7 @@
         <v>CHM-0170</v>
       </c>
       <c r="C171" s="12" t="s">
-        <v>7</v>
+        <v>217</v>
       </c>
       <c r="D171" s="12" t="str">
         <v>acetate 5.0</v>
@@ -6353,7 +6356,7 @@
         <v>CHM-0171</v>
       </c>
       <c r="C172" s="12" t="s">
-        <v>7</v>
+        <v>217</v>
       </c>
       <c r="D172" s="12" t="str">
         <v>Acetate 5.5</v>
@@ -7255,8 +7258,8 @@
       <c r="B199" s="12" t="str">
         <v>CHM-0198</v>
       </c>
-      <c r="C199" s="12" t="str">
-        <v>Biacore</v>
+      <c r="C199" s="12" t="s">
+        <v>217</v>
       </c>
       <c r="D199" s="12" t="str">
         <v>Ethanolamine-HCL</v>
@@ -7464,7 +7467,7 @@
         <v>CHM-0204</v>
       </c>
       <c r="C205" s="12" t="s">
-        <v>7</v>
+        <v>217</v>
       </c>
       <c r="D205" s="12" t="str">
         <v>Glycine 1.5</v>
@@ -7495,7 +7498,7 @@
         <v>CHM-0205</v>
       </c>
       <c r="C206" s="12" t="s">
-        <v>7</v>
+        <v>217</v>
       </c>
       <c r="D206" s="12" t="str">
         <v>Glycine 2.0</v>
@@ -7526,7 +7529,7 @@
         <v>CHM-0206</v>
       </c>
       <c r="C207" s="12" t="s">
-        <v>7</v>
+        <v>217</v>
       </c>
       <c r="D207" s="12" t="str">
         <v>Glycine 2.5</v>
@@ -7588,7 +7591,7 @@
         <v>CHM-0208</v>
       </c>
       <c r="C209" s="12" t="s">
-        <v>7</v>
+        <v>217</v>
       </c>
       <c r="D209" s="12" t="str">
         <v>HBS-EP buffer</v>
@@ -8865,7 +8868,7 @@
         <v>CHM-0247</v>
       </c>
       <c r="C248" s="12" t="s">
-        <v>7</v>
+        <v>217</v>
       </c>
       <c r="D248" s="12" t="str">
         <v>Sensor chip CM5</v>

</xml_diff>